<commit_message>
Editor de partidos en el Calendario y nombres oficiales de equipos
Boton Editar en cada partido: corrige jornada, fecha, hora, equipos,
marcador, goleadores y tarjetas. Nombres segun el afiche: Peñarol F.C
y Santa Ana F.C.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/COPA PALERMO - BASE DE DATOS (plantilla).xlsx
+++ b/descargas/COPA PALERMO - BASE DE DATOS (plantilla).xlsx
@@ -256,7 +256,7 @@
     <t>LOS RIOS</t>
   </si>
   <si>
-    <t>SANTANA F.C</t>
+    <t>SANTA ANA F.C</t>
   </si>
   <si>
     <t>GRUPO B</t>
@@ -265,7 +265,7 @@
     <t>CLUB GAROFALOS</t>
   </si>
   <si>
-    <t>PEÑAZOL F.C</t>
+    <t>PEÑAROL F.C</t>
   </si>
   <si>
     <t>MAGIC</t>

</xml_diff>

<commit_message>
Fases finales: clasifican todos y primera ronda de muerte subita
Soporta CLASIFICAN_POR_GRUPO = TODOS, cruza el 1.o de A con el ultimo de B
y nombra la ronda segun cuantos equipos juegan (muerte subita, octavos...).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/descargas/COPA PALERMO - BASE DE DATOS (plantilla).xlsx
+++ b/descargas/COPA PALERMO - BASE DE DATOS (plantilla).xlsx
@@ -52,7 +52,7 @@
     <t>-  El ID del partido (P001, P002, ...) es la llave que une PARTIDOS con GOLES y TARJETAS.</t>
   </si>
   <si>
-    <t>-  Fases finales: columna FASE = CUARTOS, SEMIFINAL, TERCER PUESTO o FINAL (no entran en la tabla de posiciones).</t>
+    <t>-  Fases finales: columna FASE = MUERTE SUBITA, OCTAVOS, CUARTOS, SEMIFINAL, TERCER PUESTO o FINAL (no entran en la tabla de posiciones).</t>
   </si>
   <si>
     <t>CATEGORIAS</t>
@@ -127,10 +127,10 @@
     <t>CLASIFICAN_POR_GRUPO</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>Cuantos pasan a fases finales por cada grupo (4 + 4 = cuartos de final)</t>
+    <t>TODOS</t>
+  </si>
+  <si>
+    <t>Cuantos pasan a fases finales por cada grupo: un numero, o TODOS si clasifican todos</t>
   </si>
   <si>
     <t>DESEMPATE</t>
@@ -1988,10 +1988,10 @@
       <formula1>"GRUPO A,GRUPO B"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C10:C400">
-      <formula1>"GRUPOS,CUARTOS,SEMIFINAL,TERCER PUESTO,FINAL"</formula1>
+      <formula1>"GRUPOS,MUERTE SUBITA,OCTAVOS,CUARTOS,SEMIFINAL,TERCER PUESTO,FINAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="C2:C400">
-      <formula1>"GRUPOS,CUARTOS,SEMIFINAL,TERCER PUESTO,FINAL"</formula1>
+      <formula1>"GRUPOS,MUERTE SUBITA,OCTAVOS,CUARTOS,SEMIFINAL,TERCER PUESTO,FINAL"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="L10:L400">
       <formula1>"PENDIENTE,JUGADO,WO LOCAL,WO VISITA,SUSPENDIDO"</formula1>

</xml_diff>